<commit_message>
Poprawa danych z excela
</commit_message>
<xml_diff>
--- a/mieszkania.xlsx
+++ b/mieszkania.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mateu\Desktop\BlockViewDesktop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0063D5FA-5D4D-4017-98FF-AA2A6A909D25}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9D090802-9B8D-47C2-8043-BEE33BE5C256}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="356" uniqueCount="226">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="288" uniqueCount="222">
   <si>
     <t>id</t>
   </si>
@@ -55,9 +55,6 @@
     <t>apt-1</t>
   </si>
   <si>
-    <t>350 000</t>
-  </si>
-  <si>
     <t>apt-2</t>
   </si>
   <si>
@@ -268,27 +265,15 @@
     <t>R100/01</t>
   </si>
   <si>
-    <t>75.42</t>
-  </si>
-  <si>
     <t>R100/02</t>
   </si>
   <si>
-    <t>53.66</t>
-  </si>
-  <si>
     <t>R100/03</t>
   </si>
   <si>
-    <t>40.52</t>
-  </si>
-  <si>
     <t>R100/04</t>
   </si>
   <si>
-    <t>56.4</t>
-  </si>
-  <si>
     <t>R100/05</t>
   </si>
   <si>
@@ -698,13 +683,19 @@
   </si>
   <si>
     <t>static\karty-lokali\R101\R101_16_L.pdf</t>
+  </si>
+  <si>
+    <t>price/meter</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="#,##0.00\ &quot;zł&quot;"/>
+  </numFmts>
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -712,8 +703,30 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="14"/>
+      <color theme="0"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <charset val="238"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color theme="0"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <charset val="238"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color theme="0"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <charset val="238"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -722,12 +735,18 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF92D050"/>
+        <fgColor rgb="FF0B5637"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF01351F"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -735,45 +754,79 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyProtection="1">
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="3" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyProtection="1">
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="3" fontId="2" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="4" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyProtection="1">
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="3" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normalny" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="6">
+    <dxf>
+      <font>
+        <color rgb="FF00B050"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFFF0000"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFFFC000"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFFF0000"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF00B050"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF00B050"/>
+      </font>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleMedium4"/>
+  <colors>
+    <mruColors>
+      <color rgb="FF0B5637"/>
+      <color rgb="FF01351F"/>
+    </mruColors>
+  </colors>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -1107,58 +1160,66 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K70"/>
+  <dimension ref="A1:L70"/>
   <sheetFormatPr defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="13.69921875" customWidth="1"/>
     <col min="2" max="2" width="13.796875" customWidth="1"/>
-    <col min="6" max="6" width="37.296875" customWidth="1"/>
-    <col min="9" max="9" width="12" customWidth="1"/>
-    <col min="10" max="10" width="9.8984375" customWidth="1"/>
-    <col min="11" max="11" width="11.19921875" customWidth="1"/>
+    <col min="3" max="3" width="4.3984375" customWidth="1"/>
+    <col min="4" max="4" width="4.5" customWidth="1"/>
+    <col min="5" max="5" width="6.3984375" customWidth="1"/>
+    <col min="6" max="6" width="41.69921875" customWidth="1"/>
+    <col min="7" max="7" width="10.69921875" customWidth="1"/>
+    <col min="8" max="8" width="13" customWidth="1"/>
+    <col min="9" max="10" width="18.59765625" customWidth="1"/>
+    <col min="11" max="11" width="9.8984375" customWidth="1"/>
+    <col min="12" max="12" width="14.296875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A1" s="4" t="s">
+    <row r="1" spans="1:12" ht="51.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="4" t="s">
+      <c r="B1" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="4" t="s">
+      <c r="C1" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="4" t="s">
+      <c r="D1" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="4" t="s">
+      <c r="E1" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="4" t="s">
+      <c r="F1" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="4" t="s">
+      <c r="G1" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="4" t="s">
+      <c r="H1" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="4" t="s">
+      <c r="I1" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="4" t="s">
-        <v>151</v>
-      </c>
-      <c r="K1" s="4" t="s">
+      <c r="J1" s="5" t="s">
+        <v>221</v>
+      </c>
+      <c r="K1" s="5" t="s">
+        <v>146</v>
+      </c>
+      <c r="L1" s="5" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:12" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C2" s="1">
         <v>255</v>
@@ -1169,31 +1230,34 @@
       <c r="E2" s="1">
         <v>111</v>
       </c>
-      <c r="F2" s="1" t="s">
-        <v>157</v>
-      </c>
-      <c r="G2" s="2" t="s">
-        <v>82</v>
+      <c r="F2" s="3" t="s">
+        <v>152</v>
+      </c>
+      <c r="G2" s="7">
+        <v>75.13</v>
       </c>
       <c r="H2" s="2">
         <v>4</v>
       </c>
-      <c r="I2" s="5">
+      <c r="I2" s="6">
         <v>894047</v>
       </c>
       <c r="J2" s="6">
+        <v>11900</v>
+      </c>
+      <c r="K2" s="4">
         <v>65</v>
       </c>
-      <c r="K2" s="2" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L2" s="2" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="3" spans="1:12" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="C3" s="1">
         <v>255</v>
@@ -1204,31 +1268,34 @@
       <c r="E3" s="1">
         <v>111</v>
       </c>
-      <c r="F3" s="1" t="s">
-        <v>158</v>
-      </c>
-      <c r="G3" s="2" t="s">
-        <v>84</v>
+      <c r="F3" s="3" t="s">
+        <v>153</v>
+      </c>
+      <c r="G3" s="7">
+        <v>53.66</v>
       </c>
       <c r="H3" s="2">
         <v>3</v>
       </c>
-      <c r="I3" s="5">
+      <c r="I3" s="6">
         <v>665384</v>
       </c>
       <c r="J3" s="6">
+        <v>12400</v>
+      </c>
+      <c r="K3" s="4">
         <v>49</v>
       </c>
-      <c r="K3" s="2" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L3" s="2" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="C4" s="1">
         <v>255</v>
@@ -1239,31 +1306,34 @@
       <c r="E4" s="1">
         <v>111</v>
       </c>
-      <c r="F4" s="1" t="s">
-        <v>159</v>
-      </c>
-      <c r="G4" s="2" t="s">
-        <v>86</v>
+      <c r="F4" s="3" t="s">
+        <v>154</v>
+      </c>
+      <c r="G4" s="7">
+        <v>40.520000000000003</v>
       </c>
       <c r="H4" s="2">
         <v>2</v>
       </c>
-      <c r="I4" s="5">
+      <c r="I4" s="6">
         <v>522708</v>
       </c>
       <c r="J4" s="6">
+        <v>12900</v>
+      </c>
+      <c r="K4" s="4">
         <v>50</v>
       </c>
-      <c r="K4" s="2" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L4" s="2" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>87</v>
+        <v>83</v>
       </c>
       <c r="C5" s="1">
         <v>255</v>
@@ -1274,31 +1344,34 @@
       <c r="E5" s="1">
         <v>111</v>
       </c>
-      <c r="F5" s="1" t="s">
-        <v>160</v>
-      </c>
-      <c r="G5" s="2" t="s">
-        <v>88</v>
+      <c r="F5" s="3" t="s">
+        <v>155</v>
+      </c>
+      <c r="G5" s="7">
+        <v>56.4</v>
       </c>
       <c r="H5" s="2">
         <v>3</v>
       </c>
-      <c r="I5" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="J5" s="1">
+      <c r="I5" s="6">
+        <v>688080</v>
+      </c>
+      <c r="J5" s="6">
+        <v>12200</v>
+      </c>
+      <c r="K5" s="1">
         <v>49</v>
       </c>
-      <c r="K5" s="2" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L5" s="2" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="6" spans="1:12" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>89</v>
+        <v>84</v>
       </c>
       <c r="C6" s="1">
         <v>255</v>
@@ -1309,31 +1382,34 @@
       <c r="E6" s="1">
         <v>111</v>
       </c>
-      <c r="F6" s="1" t="s">
-        <v>161</v>
-      </c>
-      <c r="G6" s="2">
-        <v>50</v>
+      <c r="F6" s="3" t="s">
+        <v>156</v>
+      </c>
+      <c r="G6" s="7">
+        <v>56.4</v>
       </c>
       <c r="H6" s="2">
-        <v>2</v>
-      </c>
-      <c r="I6" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="J6" s="1">
+        <v>3</v>
+      </c>
+      <c r="I6" s="6">
+        <v>688080</v>
+      </c>
+      <c r="J6" s="6">
+        <v>12200</v>
+      </c>
+      <c r="K6" s="1">
         <v>47</v>
       </c>
-      <c r="K6" s="2" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L6" s="2" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="7" spans="1:12" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="1" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>90</v>
+        <v>85</v>
       </c>
       <c r="C7" s="1">
         <v>255</v>
@@ -1344,31 +1420,34 @@
       <c r="E7" s="1">
         <v>111</v>
       </c>
-      <c r="F7" s="1" t="s">
-        <v>162</v>
-      </c>
-      <c r="G7" s="2">
-        <v>50</v>
+      <c r="F7" s="3" t="s">
+        <v>157</v>
+      </c>
+      <c r="G7" s="7">
+        <v>37.409999999999997</v>
       </c>
       <c r="H7" s="2">
         <v>2</v>
       </c>
-      <c r="I7" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="J7" s="1">
+      <c r="I7" s="6">
+        <v>490071</v>
+      </c>
+      <c r="J7" s="6">
+        <v>13100</v>
+      </c>
+      <c r="K7" s="1">
         <v>47</v>
       </c>
-      <c r="K7" s="2" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L7" s="2" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="8" spans="1:12" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>91</v>
+        <v>86</v>
       </c>
       <c r="C8" s="1">
         <v>255</v>
@@ -1379,31 +1458,34 @@
       <c r="E8" s="1">
         <v>111</v>
       </c>
-      <c r="F8" s="1" t="s">
-        <v>163</v>
-      </c>
-      <c r="G8" s="2">
-        <v>50</v>
+      <c r="F8" s="3" t="s">
+        <v>158</v>
+      </c>
+      <c r="G8" s="7">
+        <v>64.209999999999994</v>
       </c>
       <c r="H8" s="2">
-        <v>2</v>
-      </c>
-      <c r="I8" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="J8" s="1">
+        <v>3</v>
+      </c>
+      <c r="I8" s="6">
+        <v>783362</v>
+      </c>
+      <c r="J8" s="6">
+        <v>12200</v>
+      </c>
+      <c r="K8" s="1">
         <v>27</v>
       </c>
-      <c r="K8" s="2" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L8" s="2" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="9" spans="1:12" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="1" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>92</v>
+        <v>87</v>
       </c>
       <c r="C9" s="1">
         <v>111</v>
@@ -1414,31 +1496,34 @@
       <c r="E9" s="1">
         <v>246</v>
       </c>
-      <c r="F9" s="1" t="s">
-        <v>164</v>
-      </c>
-      <c r="G9" s="2">
-        <v>50</v>
+      <c r="F9" s="3" t="s">
+        <v>159</v>
+      </c>
+      <c r="G9" s="7">
+        <v>53.48</v>
       </c>
       <c r="H9" s="2">
-        <v>2</v>
-      </c>
-      <c r="I9" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="J9" s="1">
+        <v>3</v>
+      </c>
+      <c r="I9" s="6">
+        <v>668500</v>
+      </c>
+      <c r="J9" s="6">
+        <v>12500</v>
+      </c>
+      <c r="K9" s="1">
         <v>16</v>
       </c>
-      <c r="K9" s="2" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L9" s="2" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="10" spans="1:12" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="1" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>93</v>
+        <v>88</v>
       </c>
       <c r="C10" s="1">
         <v>112</v>
@@ -1449,31 +1534,34 @@
       <c r="E10" s="1">
         <v>235</v>
       </c>
-      <c r="F10" s="1" t="s">
-        <v>165</v>
-      </c>
-      <c r="G10" s="2">
-        <v>50</v>
+      <c r="F10" s="3" t="s">
+        <v>160</v>
+      </c>
+      <c r="G10" s="7">
+        <v>55.63</v>
       </c>
       <c r="H10" s="2">
-        <v>2</v>
-      </c>
-      <c r="I10" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="J10" s="1">
+        <v>3</v>
+      </c>
+      <c r="I10" s="6">
+        <v>689812</v>
+      </c>
+      <c r="J10" s="6">
+        <v>12400</v>
+      </c>
+      <c r="K10" s="1">
         <v>10</v>
       </c>
-      <c r="K10" s="2" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L10" s="2" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="11" spans="1:12" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="1" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>97</v>
+        <v>92</v>
       </c>
       <c r="C11" s="1">
         <v>111</v>
@@ -1484,31 +1572,34 @@
       <c r="E11" s="1">
         <v>223</v>
       </c>
-      <c r="F11" s="1" t="s">
-        <v>166</v>
-      </c>
-      <c r="G11" s="2">
-        <v>50</v>
+      <c r="F11" s="3" t="s">
+        <v>161</v>
+      </c>
+      <c r="G11" s="7">
+        <v>66.87</v>
       </c>
       <c r="H11" s="2">
+        <v>4</v>
+      </c>
+      <c r="I11" s="6">
+        <v>809127</v>
+      </c>
+      <c r="J11" s="6">
+        <v>12100</v>
+      </c>
+      <c r="K11" s="1">
         <v>2</v>
       </c>
-      <c r="I11" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="J11" s="1">
-        <v>2</v>
-      </c>
-      <c r="K11" s="2" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L11" s="2" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="12" spans="1:12" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="1" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>96</v>
+        <v>91</v>
       </c>
       <c r="C12" s="1">
         <v>112</v>
@@ -1519,31 +1610,34 @@
       <c r="E12" s="1">
         <v>206</v>
       </c>
-      <c r="F12" s="1" t="s">
-        <v>167</v>
-      </c>
-      <c r="G12" s="2">
-        <v>50</v>
+      <c r="F12" s="3" t="s">
+        <v>162</v>
+      </c>
+      <c r="G12" s="7">
+        <v>74.23</v>
       </c>
       <c r="H12" s="2">
-        <v>2</v>
-      </c>
-      <c r="I12" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="J12" s="1">
+        <v>4</v>
+      </c>
+      <c r="I12" s="6">
+        <v>898183</v>
+      </c>
+      <c r="J12" s="6">
+        <v>12100</v>
+      </c>
+      <c r="K12" s="1">
         <v>104</v>
       </c>
-      <c r="K12" s="2" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L12" s="2" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="13" spans="1:12" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="1" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>95</v>
+        <v>90</v>
       </c>
       <c r="C13" s="1">
         <v>111</v>
@@ -1554,31 +1648,34 @@
       <c r="E13" s="1">
         <v>181</v>
       </c>
-      <c r="F13" s="1" t="s">
-        <v>168</v>
-      </c>
-      <c r="G13" s="2">
-        <v>50</v>
+      <c r="F13" s="3" t="s">
+        <v>163</v>
+      </c>
+      <c r="G13" s="7">
+        <v>56.42</v>
       </c>
       <c r="H13" s="2">
-        <v>2</v>
-      </c>
-      <c r="I13" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="J13" s="1">
+        <v>3</v>
+      </c>
+      <c r="I13" s="6">
+        <v>693966</v>
+      </c>
+      <c r="J13" s="6">
+        <v>12300</v>
+      </c>
+      <c r="K13" s="1">
         <v>98</v>
       </c>
-      <c r="K13" s="2" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L13" s="2" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="14" spans="1:12" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="1" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>94</v>
+        <v>89</v>
       </c>
       <c r="C14" s="1">
         <v>111</v>
@@ -1589,31 +1686,34 @@
       <c r="E14" s="1">
         <v>112</v>
       </c>
-      <c r="F14" s="1" t="s">
-        <v>169</v>
-      </c>
-      <c r="G14" s="2">
-        <v>50</v>
+      <c r="F14" s="3" t="s">
+        <v>164</v>
+      </c>
+      <c r="G14" s="7">
+        <v>54.93</v>
       </c>
       <c r="H14" s="2">
-        <v>2</v>
-      </c>
-      <c r="I14" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="J14" s="1">
+        <v>3</v>
+      </c>
+      <c r="I14" s="6">
+        <v>681132</v>
+      </c>
+      <c r="J14" s="6">
+        <v>12400</v>
+      </c>
+      <c r="K14" s="1">
         <v>107</v>
       </c>
-      <c r="K14" s="2" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L14" s="2" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="15" spans="1:12" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>98</v>
+        <v>93</v>
       </c>
       <c r="C15" s="1">
         <v>181</v>
@@ -1624,31 +1724,34 @@
       <c r="E15" s="1">
         <v>111</v>
       </c>
-      <c r="F15" s="1" t="s">
-        <v>170</v>
-      </c>
-      <c r="G15" s="2">
-        <v>50</v>
+      <c r="F15" s="3" t="s">
+        <v>165</v>
+      </c>
+      <c r="G15" s="7">
+        <v>37.4</v>
       </c>
       <c r="H15" s="2">
         <v>2</v>
       </c>
-      <c r="I15" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="J15" s="1">
+      <c r="I15" s="6">
+        <v>493680</v>
+      </c>
+      <c r="J15" s="6">
+        <v>13200</v>
+      </c>
+      <c r="K15" s="1">
         <v>109</v>
       </c>
-      <c r="K15" s="2" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L15" s="2" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="16" spans="1:12" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="1" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>99</v>
+        <v>94</v>
       </c>
       <c r="C16" s="1">
         <v>206</v>
@@ -1659,31 +1762,34 @@
       <c r="E16" s="1">
         <v>111</v>
       </c>
-      <c r="F16" s="1" t="s">
-        <v>171</v>
-      </c>
-      <c r="G16" s="2">
-        <v>50</v>
+      <c r="F16" s="3" t="s">
+        <v>166</v>
+      </c>
+      <c r="G16" s="7">
+        <v>35.950000000000003</v>
       </c>
       <c r="H16" s="2">
         <v>2</v>
       </c>
-      <c r="I16" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="J16" s="1">
+      <c r="I16" s="6">
+        <v>474540</v>
+      </c>
+      <c r="J16" s="6">
+        <v>13200</v>
+      </c>
+      <c r="K16" s="1">
         <v>114</v>
       </c>
-      <c r="K16" s="2" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="17" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L16" s="2" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="17" spans="1:12" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="1" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>100</v>
+        <v>95</v>
       </c>
       <c r="C17" s="1">
         <v>223</v>
@@ -1694,31 +1800,34 @@
       <c r="E17" s="1">
         <v>111</v>
       </c>
-      <c r="F17" s="1" t="s">
-        <v>172</v>
-      </c>
-      <c r="G17" s="2">
-        <v>50</v>
+      <c r="F17" s="3" t="s">
+        <v>167</v>
+      </c>
+      <c r="G17" s="7">
+        <v>54.47</v>
       </c>
       <c r="H17" s="2">
-        <v>2</v>
-      </c>
-      <c r="I17" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="J17" s="1">
+        <v>3</v>
+      </c>
+      <c r="I17" s="6">
+        <v>675428</v>
+      </c>
+      <c r="J17" s="6">
+        <v>12400</v>
+      </c>
+      <c r="K17" s="1">
         <v>114</v>
       </c>
-      <c r="K17" s="2" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="18" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L17" s="2" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="18" spans="1:12" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="1" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>101</v>
+        <v>96</v>
       </c>
       <c r="C18" s="1">
         <v>236</v>
@@ -1729,31 +1838,34 @@
       <c r="E18" s="1">
         <v>111</v>
       </c>
-      <c r="F18" s="1" t="s">
-        <v>173</v>
-      </c>
-      <c r="G18" s="2">
-        <v>50</v>
+      <c r="F18" s="3" t="s">
+        <v>168</v>
+      </c>
+      <c r="G18" s="7">
+        <v>66.45</v>
       </c>
       <c r="H18" s="2">
-        <v>2</v>
-      </c>
-      <c r="I18" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="J18" s="1">
+        <v>4</v>
+      </c>
+      <c r="I18" s="6">
+        <v>804045</v>
+      </c>
+      <c r="J18" s="6">
+        <v>12100</v>
+      </c>
+      <c r="K18" s="1">
         <v>119</v>
       </c>
-      <c r="K18" s="2" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="19" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L18" s="2" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="19" spans="1:12" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="1" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>102</v>
+        <v>97</v>
       </c>
       <c r="C19" s="1">
         <v>246</v>
@@ -1764,31 +1876,34 @@
       <c r="E19" s="1">
         <v>111</v>
       </c>
-      <c r="F19" s="1" t="s">
-        <v>174</v>
-      </c>
-      <c r="G19" s="2">
-        <v>50</v>
+      <c r="F19" s="3" t="s">
+        <v>169</v>
+      </c>
+      <c r="G19" s="7">
+        <v>74.39</v>
       </c>
       <c r="H19" s="2">
-        <v>2</v>
-      </c>
-      <c r="I19" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="J19" s="1">
+        <v>4</v>
+      </c>
+      <c r="I19" s="6">
+        <v>900119</v>
+      </c>
+      <c r="J19" s="6">
+        <v>12100</v>
+      </c>
+      <c r="K19" s="1">
         <v>90</v>
       </c>
-      <c r="K19" s="2" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="20" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L19" s="2" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="20" spans="1:12" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A20" s="1" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>103</v>
+        <v>98</v>
       </c>
       <c r="C20" s="1">
         <v>111</v>
@@ -1799,31 +1914,34 @@
       <c r="E20" s="1">
         <v>255</v>
       </c>
-      <c r="F20" s="1" t="s">
-        <v>175</v>
-      </c>
-      <c r="G20" s="2">
-        <v>50</v>
+      <c r="F20" s="3" t="s">
+        <v>170</v>
+      </c>
+      <c r="G20" s="7">
+        <v>75.319999999999993</v>
       </c>
       <c r="H20" s="2">
-        <v>2</v>
-      </c>
-      <c r="I20" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="J20" s="1">
+        <v>4</v>
+      </c>
+      <c r="I20" s="6">
+        <v>888776</v>
+      </c>
+      <c r="J20" s="6">
+        <v>11800</v>
+      </c>
+      <c r="K20" s="1">
         <v>65</v>
       </c>
-      <c r="K20" s="2" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="21" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L20" s="2" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="21" spans="1:12" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A21" s="1" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>104</v>
+        <v>99</v>
       </c>
       <c r="C21" s="1">
         <v>112</v>
@@ -1834,31 +1952,34 @@
       <c r="E21" s="1">
         <v>255</v>
       </c>
-      <c r="F21" s="1" t="s">
-        <v>176</v>
-      </c>
-      <c r="G21" s="2">
+      <c r="F21" s="3" t="s">
+        <v>171</v>
+      </c>
+      <c r="G21" s="7">
+        <v>53.66</v>
+      </c>
+      <c r="H21" s="2">
+        <v>3</v>
+      </c>
+      <c r="I21" s="6">
+        <v>665384</v>
+      </c>
+      <c r="J21" s="6">
+        <v>12400</v>
+      </c>
+      <c r="K21" s="1">
         <v>50</v>
       </c>
-      <c r="H21" s="2">
-        <v>2</v>
-      </c>
-      <c r="I21" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="J21" s="1">
-        <v>50</v>
-      </c>
-      <c r="K21" s="2" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="22" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L21" s="2" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="22" spans="1:12" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A22" s="1" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>105</v>
+        <v>100</v>
       </c>
       <c r="C22" s="1">
         <v>111</v>
@@ -1869,31 +1990,34 @@
       <c r="E22" s="1">
         <v>255</v>
       </c>
-      <c r="F22" s="1" t="s">
-        <v>177</v>
-      </c>
-      <c r="G22" s="2">
-        <v>50</v>
+      <c r="F22" s="3" t="s">
+        <v>172</v>
+      </c>
+      <c r="G22" s="7">
+        <v>40.520000000000003</v>
       </c>
       <c r="H22" s="2">
         <v>2</v>
       </c>
-      <c r="I22" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="J22" s="1">
+      <c r="I22" s="6">
+        <v>518656</v>
+      </c>
+      <c r="J22" s="6">
+        <v>12800</v>
+      </c>
+      <c r="K22" s="1">
         <v>48</v>
       </c>
-      <c r="K22" s="2" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="23" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L22" s="2" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="23" spans="1:12" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A23" s="1" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>106</v>
+        <v>101</v>
       </c>
       <c r="C23" s="1">
         <v>111</v>
@@ -1904,31 +2028,34 @@
       <c r="E23" s="1">
         <v>255</v>
       </c>
-      <c r="F23" s="1" t="s">
-        <v>178</v>
-      </c>
-      <c r="G23" s="2">
-        <v>50</v>
+      <c r="F23" s="3" t="s">
+        <v>173</v>
+      </c>
+      <c r="G23" s="7">
+        <v>56.4</v>
       </c>
       <c r="H23" s="2">
-        <v>2</v>
-      </c>
-      <c r="I23" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="J23" s="1">
+        <v>3</v>
+      </c>
+      <c r="I23" s="6">
+        <v>688080</v>
+      </c>
+      <c r="J23" s="6">
+        <v>12200</v>
+      </c>
+      <c r="K23" s="1">
         <v>48</v>
       </c>
-      <c r="K23" s="2" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="24" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L23" s="2" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="24" spans="1:12" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A24" s="1" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>107</v>
+        <v>102</v>
       </c>
       <c r="C24" s="1">
         <v>112</v>
@@ -1939,31 +2066,34 @@
       <c r="E24" s="1">
         <v>255</v>
       </c>
-      <c r="F24" s="1" t="s">
-        <v>179</v>
-      </c>
-      <c r="G24" s="2">
-        <v>50</v>
+      <c r="F24" s="3" t="s">
+        <v>174</v>
+      </c>
+      <c r="G24" s="7">
+        <v>56.4</v>
       </c>
       <c r="H24" s="2">
-        <v>2</v>
-      </c>
-      <c r="I24" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="J24" s="1">
+        <v>3</v>
+      </c>
+      <c r="I24" s="6">
+        <v>688080</v>
+      </c>
+      <c r="J24" s="6">
+        <v>12200</v>
+      </c>
+      <c r="K24" s="1">
         <v>47</v>
       </c>
-      <c r="K24" s="2" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="25" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L24" s="2" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="25" spans="1:12" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A25" s="1" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>108</v>
+        <v>103</v>
       </c>
       <c r="C25" s="1">
         <v>111</v>
@@ -1974,31 +2104,34 @@
       <c r="E25" s="1">
         <v>255</v>
       </c>
-      <c r="F25" s="1" t="s">
-        <v>180</v>
-      </c>
-      <c r="G25" s="2">
-        <v>50</v>
+      <c r="F25" s="3" t="s">
+        <v>175</v>
+      </c>
+      <c r="G25" s="7">
+        <v>58.86</v>
       </c>
       <c r="H25" s="2">
-        <v>2</v>
-      </c>
-      <c r="I25" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="J25" s="1">
+        <v>3</v>
+      </c>
+      <c r="I25" s="6">
+        <v>718092</v>
+      </c>
+      <c r="J25" s="6">
+        <v>12200</v>
+      </c>
+      <c r="K25" s="1">
         <v>43</v>
       </c>
-      <c r="K25" s="2" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="26" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L25" s="2" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="26" spans="1:12" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A26" s="1" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>109</v>
+        <v>104</v>
       </c>
       <c r="C26" s="1">
         <v>111</v>
@@ -2009,31 +2142,34 @@
       <c r="E26" s="1">
         <v>255</v>
       </c>
-      <c r="F26" s="1" t="s">
-        <v>181</v>
-      </c>
-      <c r="G26" s="2">
-        <v>50</v>
+      <c r="F26" s="3" t="s">
+        <v>176</v>
+      </c>
+      <c r="G26" s="7">
+        <v>60.69</v>
       </c>
       <c r="H26" s="2">
-        <v>2</v>
-      </c>
-      <c r="I26" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="J26" s="1">
+        <v>3</v>
+      </c>
+      <c r="I26" s="6">
+        <v>740418</v>
+      </c>
+      <c r="J26" s="6">
+        <v>12200</v>
+      </c>
+      <c r="K26" s="1">
         <v>27</v>
       </c>
-      <c r="K26" s="2" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="27" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L26" s="2" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="27" spans="1:12" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A27" s="1" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>110</v>
+        <v>105</v>
       </c>
       <c r="C27" s="1">
         <v>223</v>
@@ -2044,31 +2180,34 @@
       <c r="E27" s="1">
         <v>111</v>
       </c>
-      <c r="F27" s="1" t="s">
-        <v>219</v>
-      </c>
-      <c r="G27" s="2">
+      <c r="F27" s="3" t="s">
+        <v>214</v>
+      </c>
+      <c r="G27" s="7">
+        <v>50.49</v>
+      </c>
+      <c r="H27" s="2">
+        <v>3</v>
+      </c>
+      <c r="I27" s="6">
+        <v>631125</v>
+      </c>
+      <c r="J27" s="6">
+        <v>12500</v>
+      </c>
+      <c r="K27" s="1">
+        <v>17</v>
+      </c>
+      <c r="L27" s="2" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="28" spans="1:12" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A28" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="H27" s="2">
-        <v>2</v>
-      </c>
-      <c r="I27" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="J27" s="1">
-        <v>17</v>
-      </c>
-      <c r="K27" s="2" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="28" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A28" s="1" t="s">
-        <v>51</v>
-      </c>
       <c r="B28" s="2" t="s">
-        <v>111</v>
+        <v>106</v>
       </c>
       <c r="C28" s="1">
         <v>255</v>
@@ -2079,31 +2218,34 @@
       <c r="E28" s="1">
         <v>181</v>
       </c>
-      <c r="F28" s="1" t="s">
-        <v>220</v>
-      </c>
-      <c r="G28" s="2">
-        <v>50</v>
+      <c r="F28" s="3" t="s">
+        <v>215</v>
+      </c>
+      <c r="G28" s="7">
+        <v>52.48</v>
       </c>
       <c r="H28" s="2">
-        <v>2</v>
-      </c>
-      <c r="I28" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="J28" s="1">
+        <v>3</v>
+      </c>
+      <c r="I28" s="6">
+        <v>656000</v>
+      </c>
+      <c r="J28" s="6">
+        <v>12500</v>
+      </c>
+      <c r="K28" s="1">
         <v>15</v>
       </c>
-      <c r="K28" s="2" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="29" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L28" s="2" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="29" spans="1:12" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A29" s="1" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>112</v>
+        <v>107</v>
       </c>
       <c r="C29" s="1">
         <v>255</v>
@@ -2114,31 +2256,34 @@
       <c r="E29" s="1">
         <v>206</v>
       </c>
-      <c r="F29" s="1" t="s">
-        <v>182</v>
-      </c>
-      <c r="G29" s="2">
-        <v>50</v>
+      <c r="F29" s="3" t="s">
+        <v>177</v>
+      </c>
+      <c r="G29" s="7">
+        <v>67.05</v>
       </c>
       <c r="H29" s="2">
-        <v>2</v>
-      </c>
-      <c r="I29" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="J29" s="1">
+        <v>4</v>
+      </c>
+      <c r="I29" s="6">
+        <v>811305</v>
+      </c>
+      <c r="J29" s="6">
+        <v>12100</v>
+      </c>
+      <c r="K29" s="1">
         <v>3</v>
       </c>
-      <c r="K29" s="2" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="30" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L29" s="2" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="30" spans="1:12" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A30" s="1" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>113</v>
+        <v>108</v>
       </c>
       <c r="C30" s="1">
         <v>255</v>
@@ -2149,31 +2294,34 @@
       <c r="E30" s="1">
         <v>223</v>
       </c>
-      <c r="F30" s="1" t="s">
-        <v>183</v>
-      </c>
-      <c r="G30" s="2">
-        <v>50</v>
+      <c r="F30" s="3" t="s">
+        <v>178</v>
+      </c>
+      <c r="G30" s="7">
+        <v>74.23</v>
       </c>
       <c r="H30" s="2">
-        <v>2</v>
-      </c>
-      <c r="I30" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="J30" s="1">
+        <v>4</v>
+      </c>
+      <c r="I30" s="6">
+        <v>883337</v>
+      </c>
+      <c r="J30" s="6">
+        <v>11900</v>
+      </c>
+      <c r="K30" s="1">
         <v>95</v>
       </c>
-      <c r="K30" s="2" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="31" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L30" s="2" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="31" spans="1:12" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A31" s="1" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>114</v>
+        <v>109</v>
       </c>
       <c r="C31" s="1">
         <v>255</v>
@@ -2184,31 +2332,34 @@
       <c r="E31" s="1">
         <v>235</v>
       </c>
-      <c r="F31" s="1" t="s">
-        <v>221</v>
-      </c>
-      <c r="G31" s="2">
-        <v>50</v>
+      <c r="F31" s="3" t="s">
+        <v>216</v>
+      </c>
+      <c r="G31" s="7">
+        <v>52.61</v>
       </c>
       <c r="H31" s="2">
-        <v>2</v>
-      </c>
-      <c r="I31" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="J31" s="1">
+        <v>3</v>
+      </c>
+      <c r="I31" s="6">
+        <v>657625</v>
+      </c>
+      <c r="J31" s="6">
+        <v>12500</v>
+      </c>
+      <c r="K31" s="1">
         <v>105</v>
       </c>
-      <c r="K31" s="2" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="32" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L31" s="2" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="32" spans="1:12" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A32" s="1" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>115</v>
+        <v>110</v>
       </c>
       <c r="C32" s="1">
         <v>255</v>
@@ -2219,31 +2370,34 @@
       <c r="E32" s="1">
         <v>247</v>
       </c>
-      <c r="F32" s="1" t="s">
-        <v>222</v>
-      </c>
-      <c r="G32" s="2">
-        <v>50</v>
+      <c r="F32" s="3" t="s">
+        <v>217</v>
+      </c>
+      <c r="G32" s="7">
+        <v>52.15</v>
       </c>
       <c r="H32" s="2">
-        <v>2</v>
-      </c>
-      <c r="I32" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="J32" s="1">
+        <v>3</v>
+      </c>
+      <c r="I32" s="6">
+        <v>651875</v>
+      </c>
+      <c r="J32" s="6">
+        <v>12500</v>
+      </c>
+      <c r="K32" s="1">
         <v>107</v>
       </c>
-      <c r="K32" s="2" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="33" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L32" s="2" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="33" spans="1:12" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A33" s="1" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B33" s="2" t="s">
-        <v>116</v>
+        <v>111</v>
       </c>
       <c r="C33" s="1">
         <v>255</v>
@@ -2254,31 +2408,34 @@
       <c r="E33" s="1">
         <v>255</v>
       </c>
-      <c r="F33" s="1" t="s">
-        <v>223</v>
-      </c>
-      <c r="G33" s="2">
-        <v>50</v>
+      <c r="F33" s="3" t="s">
+        <v>218</v>
+      </c>
+      <c r="G33" s="7">
+        <v>33.83</v>
       </c>
       <c r="H33" s="2">
         <v>2</v>
       </c>
-      <c r="I33" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="J33" s="1">
+      <c r="I33" s="6">
+        <v>446556</v>
+      </c>
+      <c r="J33" s="6">
+        <v>13200</v>
+      </c>
+      <c r="K33" s="1">
         <v>110</v>
       </c>
-      <c r="K33" s="2" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="34" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L33" s="2" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="34" spans="1:12" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A34" s="1" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B34" s="2" t="s">
-        <v>117</v>
+        <v>112</v>
       </c>
       <c r="C34" s="1">
         <v>247</v>
@@ -2289,31 +2446,34 @@
       <c r="E34" s="1">
         <v>255</v>
       </c>
-      <c r="F34" s="1" t="s">
-        <v>224</v>
-      </c>
-      <c r="G34" s="2">
-        <v>50</v>
+      <c r="F34" s="3" t="s">
+        <v>219</v>
+      </c>
+      <c r="G34" s="7">
+        <v>35.950000000000003</v>
       </c>
       <c r="H34" s="2">
         <v>2</v>
       </c>
-      <c r="I34" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="J34" s="1">
-        <v>111</v>
-      </c>
-      <c r="K34" s="2" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="35" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="I34" s="6">
+        <v>474540</v>
+      </c>
+      <c r="J34" s="6">
+        <v>13200</v>
+      </c>
+      <c r="K34" s="1">
+        <v>111</v>
+      </c>
+      <c r="L34" s="2" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="35" spans="1:12" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A35" s="1" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B35" s="2" t="s">
-        <v>118</v>
+        <v>113</v>
       </c>
       <c r="C35" s="1">
         <v>236</v>
@@ -2324,31 +2484,34 @@
       <c r="E35" s="1">
         <v>255</v>
       </c>
-      <c r="F35" s="1" t="s">
-        <v>225</v>
-      </c>
-      <c r="G35" s="2">
-        <v>50</v>
+      <c r="F35" s="3" t="s">
+        <v>220</v>
+      </c>
+      <c r="G35" s="7">
+        <v>51.58</v>
       </c>
       <c r="H35" s="2">
-        <v>2</v>
-      </c>
-      <c r="I35" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="J35" s="1">
         <v>3</v>
       </c>
-      <c r="K35" s="2" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="36" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="I35" s="6">
+        <v>644750</v>
+      </c>
+      <c r="J35" s="6">
+        <v>12500</v>
+      </c>
+      <c r="K35" s="1">
+        <v>3</v>
+      </c>
+      <c r="L35" s="2" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="36" spans="1:12" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A36" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B36" s="2" t="s">
-        <v>119</v>
+        <v>114</v>
       </c>
       <c r="C36" s="1">
         <v>223</v>
@@ -2359,31 +2522,34 @@
       <c r="E36" s="1">
         <v>255</v>
       </c>
-      <c r="F36" s="1" t="s">
-        <v>184</v>
-      </c>
-      <c r="G36" s="2">
-        <v>50</v>
+      <c r="F36" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="G36" s="7">
+        <v>66.66</v>
       </c>
       <c r="H36" s="2">
-        <v>2</v>
-      </c>
-      <c r="I36" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="J36" s="1">
+        <v>4</v>
+      </c>
+      <c r="I36" s="6">
+        <v>806586</v>
+      </c>
+      <c r="J36" s="6">
+        <v>12100</v>
+      </c>
+      <c r="K36" s="1">
         <v>115</v>
       </c>
-      <c r="K36" s="2" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="37" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L36" s="2" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="37" spans="1:12" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A37" s="1" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B37" s="2" t="s">
-        <v>120</v>
+        <v>115</v>
       </c>
       <c r="C37" s="1">
         <v>206</v>
@@ -2394,31 +2560,34 @@
       <c r="E37" s="1">
         <v>255</v>
       </c>
-      <c r="F37" s="1" t="s">
-        <v>185</v>
-      </c>
-      <c r="G37" s="2">
-        <v>50</v>
+      <c r="F37" s="3" t="s">
+        <v>180</v>
+      </c>
+      <c r="G37" s="7">
+        <v>93.93</v>
       </c>
       <c r="H37" s="2">
-        <v>2</v>
-      </c>
-      <c r="I37" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="J37" s="1">
+        <v>5</v>
+      </c>
+      <c r="I37" s="6">
+        <v>1108374</v>
+      </c>
+      <c r="J37" s="6">
+        <v>11800</v>
+      </c>
+      <c r="K37" s="1">
         <v>91</v>
       </c>
-      <c r="K37" s="2" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="38" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L37" s="2" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="38" spans="1:12" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A38" s="1" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="B38" s="2" t="s">
-        <v>121</v>
+        <v>116</v>
       </c>
       <c r="C38" s="1">
         <v>207</v>
@@ -2429,31 +2598,34 @@
       <c r="E38" s="1">
         <v>111</v>
       </c>
-      <c r="F38" s="1" t="s">
-        <v>186</v>
-      </c>
-      <c r="G38" s="2">
-        <v>50</v>
+      <c r="F38" s="3" t="s">
+        <v>181</v>
+      </c>
+      <c r="G38" s="7">
+        <v>75.19</v>
       </c>
       <c r="H38" s="2">
-        <v>2</v>
-      </c>
-      <c r="I38" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="J38" s="1">
+        <v>4</v>
+      </c>
+      <c r="I38" s="6">
+        <v>894761</v>
+      </c>
+      <c r="J38" s="6">
+        <v>11900</v>
+      </c>
+      <c r="K38" s="1">
         <v>65</v>
       </c>
-      <c r="K38" s="2" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="39" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L38" s="2" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="39" spans="1:12" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A39" s="1" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B39" s="2" t="s">
-        <v>122</v>
+        <v>117</v>
       </c>
       <c r="C39" s="1">
         <v>215</v>
@@ -2464,31 +2636,34 @@
       <c r="E39" s="1">
         <v>111</v>
       </c>
-      <c r="F39" s="1" t="s">
-        <v>187</v>
-      </c>
-      <c r="G39" s="2">
+      <c r="F39" s="3" t="s">
+        <v>182</v>
+      </c>
+      <c r="G39" s="7">
+        <v>53.66</v>
+      </c>
+      <c r="H39" s="2">
+        <v>3</v>
+      </c>
+      <c r="I39" s="6">
+        <v>665384</v>
+      </c>
+      <c r="J39" s="6">
+        <v>12400</v>
+      </c>
+      <c r="K39" s="1">
         <v>50</v>
       </c>
-      <c r="H39" s="2">
-        <v>2</v>
-      </c>
-      <c r="I39" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="J39" s="1">
-        <v>50</v>
-      </c>
-      <c r="K39" s="2" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="40" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L39" s="2" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="40" spans="1:12" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A40" s="1" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B40" s="2" t="s">
-        <v>123</v>
+        <v>118</v>
       </c>
       <c r="C40" s="1">
         <v>223</v>
@@ -2499,31 +2674,34 @@
       <c r="E40" s="1">
         <v>111</v>
       </c>
-      <c r="F40" s="1" t="s">
-        <v>188</v>
-      </c>
-      <c r="G40" s="2">
-        <v>50</v>
+      <c r="F40" s="3" t="s">
+        <v>183</v>
+      </c>
+      <c r="G40" s="7">
+        <v>40.57</v>
       </c>
       <c r="H40" s="2">
         <v>2</v>
       </c>
-      <c r="I40" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="J40" s="1">
+      <c r="I40" s="6">
+        <v>523353</v>
+      </c>
+      <c r="J40" s="6">
+        <v>12900</v>
+      </c>
+      <c r="K40" s="1">
         <v>50</v>
       </c>
-      <c r="K40" s="2" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="41" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L40" s="2" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="41" spans="1:12" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A41" s="1" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="B41" s="2" t="s">
-        <v>124</v>
+        <v>119</v>
       </c>
       <c r="C41" s="1">
         <v>224</v>
@@ -2534,31 +2712,34 @@
       <c r="E41" s="1">
         <v>112</v>
       </c>
-      <c r="F41" s="1" t="s">
-        <v>189</v>
-      </c>
-      <c r="G41" s="2">
-        <v>50</v>
+      <c r="F41" s="3" t="s">
+        <v>184</v>
+      </c>
+      <c r="G41" s="7">
+        <v>56.43</v>
       </c>
       <c r="H41" s="2">
-        <v>2</v>
-      </c>
-      <c r="I41" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="J41" s="1">
+        <v>3</v>
+      </c>
+      <c r="I41" s="6">
+        <v>688446</v>
+      </c>
+      <c r="J41" s="6">
+        <v>12200</v>
+      </c>
+      <c r="K41" s="1">
         <v>48</v>
       </c>
-      <c r="K41" s="2" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="42" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L41" s="2" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="42" spans="1:12" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A42" s="1" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B42" s="2" t="s">
-        <v>125</v>
+        <v>120</v>
       </c>
       <c r="C42" s="1">
         <v>223</v>
@@ -2569,31 +2750,34 @@
       <c r="E42" s="1">
         <v>111</v>
       </c>
-      <c r="F42" s="1" t="s">
-        <v>190</v>
-      </c>
-      <c r="G42" s="2">
-        <v>50</v>
+      <c r="F42" s="3" t="s">
+        <v>185</v>
+      </c>
+      <c r="G42" s="7">
+        <v>56.43</v>
       </c>
       <c r="H42" s="2">
-        <v>2</v>
-      </c>
-      <c r="I42" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="J42" s="1">
+        <v>3</v>
+      </c>
+      <c r="I42" s="6">
+        <v>688446</v>
+      </c>
+      <c r="J42" s="6">
+        <v>12200</v>
+      </c>
+      <c r="K42" s="1">
         <v>47</v>
       </c>
-      <c r="K42" s="2" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="43" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L42" s="2" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="43" spans="1:12" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A43" s="1" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B43" s="2" t="s">
-        <v>126</v>
+        <v>121</v>
       </c>
       <c r="C43" s="1">
         <v>224</v>
@@ -2604,31 +2788,34 @@
       <c r="E43" s="1">
         <v>111</v>
       </c>
-      <c r="F43" s="1" t="s">
-        <v>191</v>
-      </c>
-      <c r="G43" s="2">
-        <v>50</v>
+      <c r="F43" s="3" t="s">
+        <v>186</v>
+      </c>
+      <c r="G43" s="7">
+        <v>58.87</v>
       </c>
       <c r="H43" s="2">
-        <v>2</v>
-      </c>
-      <c r="I43" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="J43" s="1">
+        <v>3</v>
+      </c>
+      <c r="I43" s="6">
+        <v>724101</v>
+      </c>
+      <c r="J43" s="6">
+        <v>12300</v>
+      </c>
+      <c r="K43" s="1">
         <v>47</v>
       </c>
-      <c r="K43" s="2" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="44" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L43" s="2" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="44" spans="1:12" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A44" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B44" s="2" t="s">
-        <v>127</v>
+        <v>122</v>
       </c>
       <c r="C44" s="1">
         <v>223</v>
@@ -2639,31 +2826,34 @@
       <c r="E44" s="1">
         <v>111</v>
       </c>
-      <c r="F44" s="1" t="s">
-        <v>192</v>
-      </c>
-      <c r="G44" s="2">
-        <v>50</v>
+      <c r="F44" s="3" t="s">
+        <v>187</v>
+      </c>
+      <c r="G44" s="7">
+        <v>60.77</v>
       </c>
       <c r="H44" s="2">
-        <v>2</v>
-      </c>
-      <c r="I44" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="J44" s="1">
+        <v>3</v>
+      </c>
+      <c r="I44" s="6">
+        <v>741394</v>
+      </c>
+      <c r="J44" s="6">
+        <v>12200</v>
+      </c>
+      <c r="K44" s="1">
         <v>25</v>
       </c>
-      <c r="K44" s="2" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="45" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L44" s="2" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="45" spans="1:12" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A45" s="1" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B45" s="2" t="s">
-        <v>128</v>
+        <v>123</v>
       </c>
       <c r="C45" s="1">
         <v>111</v>
@@ -2674,31 +2864,34 @@
       <c r="E45" s="1">
         <v>223</v>
       </c>
-      <c r="F45" s="1" t="s">
-        <v>193</v>
-      </c>
-      <c r="G45" s="2">
-        <v>50</v>
+      <c r="F45" s="3" t="s">
+        <v>188</v>
+      </c>
+      <c r="G45" s="7">
+        <v>50.49</v>
       </c>
       <c r="H45" s="2">
-        <v>2</v>
-      </c>
-      <c r="I45" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="J45" s="1">
+        <v>3</v>
+      </c>
+      <c r="I45" s="6">
+        <v>631125</v>
+      </c>
+      <c r="J45" s="6">
+        <v>12500</v>
+      </c>
+      <c r="K45" s="1">
         <v>16</v>
       </c>
-      <c r="K45" s="2" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="46" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L45" s="2" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="46" spans="1:12" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A46" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B46" s="2" t="s">
-        <v>129</v>
+        <v>124</v>
       </c>
       <c r="C46" s="1">
         <v>112</v>
@@ -2709,31 +2902,34 @@
       <c r="E46" s="1">
         <v>224</v>
       </c>
-      <c r="F46" s="1" t="s">
-        <v>194</v>
-      </c>
-      <c r="G46" s="2">
-        <v>50</v>
+      <c r="F46" s="3" t="s">
+        <v>189</v>
+      </c>
+      <c r="G46" s="7">
+        <v>80.790000000000006</v>
       </c>
       <c r="H46" s="2">
         <v>2</v>
       </c>
-      <c r="I46" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="J46" s="1">
+      <c r="I46" s="6">
+        <v>937164</v>
+      </c>
+      <c r="J46" s="6">
+        <v>11600</v>
+      </c>
+      <c r="K46" s="1">
         <v>14</v>
       </c>
-      <c r="K46" s="2" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="47" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L46" s="2" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="47" spans="1:12" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A47" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B47" s="2" t="s">
-        <v>130</v>
+        <v>125</v>
       </c>
       <c r="C47" s="1">
         <v>112</v>
@@ -2744,31 +2940,34 @@
       <c r="E47" s="1">
         <v>223</v>
       </c>
-      <c r="F47" s="1" t="s">
-        <v>195</v>
-      </c>
-      <c r="G47" s="2">
-        <v>50</v>
+      <c r="F47" s="3" t="s">
+        <v>190</v>
+      </c>
+      <c r="G47" s="7">
+        <v>81.7</v>
       </c>
       <c r="H47" s="2">
-        <v>2</v>
-      </c>
-      <c r="I47" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="J47" s="1">
+        <v>4</v>
+      </c>
+      <c r="I47" s="6">
+        <v>972230</v>
+      </c>
+      <c r="J47" s="6">
+        <v>11900</v>
+      </c>
+      <c r="K47" s="1">
         <v>1</v>
       </c>
-      <c r="K47" s="2" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="48" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L47" s="2" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="48" spans="1:12" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A48" s="1" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B48" s="2" t="s">
-        <v>131</v>
+        <v>126</v>
       </c>
       <c r="C48" s="1">
         <v>112</v>
@@ -2779,31 +2978,34 @@
       <c r="E48" s="1">
         <v>215</v>
       </c>
-      <c r="F48" s="1" t="s">
-        <v>196</v>
-      </c>
-      <c r="G48" s="2">
-        <v>50</v>
+      <c r="F48" s="3" t="s">
+        <v>191</v>
+      </c>
+      <c r="G48" s="7">
+        <v>99.02</v>
       </c>
       <c r="H48" s="2">
-        <v>2</v>
-      </c>
-      <c r="I48" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="J48" s="1">
+        <v>3</v>
+      </c>
+      <c r="I48" s="6">
+        <v>1109024</v>
+      </c>
+      <c r="J48" s="6">
+        <v>11200</v>
+      </c>
+      <c r="K48" s="1">
         <v>92</v>
       </c>
-      <c r="K48" s="2" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="49" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L48" s="2" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="49" spans="1:12" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A49" s="1" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B49" s="2" t="s">
-        <v>132</v>
+        <v>127</v>
       </c>
       <c r="C49" s="1">
         <v>111</v>
@@ -2814,31 +3016,34 @@
       <c r="E49" s="1">
         <v>206</v>
       </c>
-      <c r="F49" s="1" t="s">
-        <v>197</v>
-      </c>
-      <c r="G49" s="2">
-        <v>50</v>
+      <c r="F49" s="3" t="s">
+        <v>192</v>
+      </c>
+      <c r="G49" s="7">
+        <v>57.32</v>
       </c>
       <c r="H49" s="2">
-        <v>2</v>
-      </c>
-      <c r="I49" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="J49" s="1">
+        <v>1</v>
+      </c>
+      <c r="I49" s="6">
+        <v>705036</v>
+      </c>
+      <c r="J49" s="6">
+        <v>12300</v>
+      </c>
+      <c r="K49" s="1">
         <v>92</v>
       </c>
-      <c r="K49" s="2" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="50" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L49" s="2" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="50" spans="1:12" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A50" s="1" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B50" s="2" t="s">
-        <v>133</v>
+        <v>128</v>
       </c>
       <c r="C50" s="1">
         <v>112</v>
@@ -2849,31 +3054,34 @@
       <c r="E50" s="1">
         <v>196</v>
       </c>
-      <c r="F50" s="1" t="s">
-        <v>198</v>
-      </c>
-      <c r="G50" s="2">
-        <v>50</v>
+      <c r="F50" s="3" t="s">
+        <v>193</v>
+      </c>
+      <c r="G50" s="7">
+        <v>52.54</v>
       </c>
       <c r="H50" s="2">
-        <v>2</v>
-      </c>
-      <c r="I50" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="J50" s="1">
+        <v>3</v>
+      </c>
+      <c r="I50" s="6">
+        <v>656750</v>
+      </c>
+      <c r="J50" s="6">
+        <v>12500</v>
+      </c>
+      <c r="K50" s="1">
         <v>94</v>
       </c>
-      <c r="K50" s="2" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="51" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L50" s="2" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="51" spans="1:12" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A51" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B51" s="2" t="s">
-        <v>134</v>
+        <v>129</v>
       </c>
       <c r="C51" s="1">
         <v>111</v>
@@ -2884,31 +3092,34 @@
       <c r="E51" s="1">
         <v>181</v>
       </c>
-      <c r="F51" s="1" t="s">
-        <v>199</v>
-      </c>
-      <c r="G51" s="2">
-        <v>50</v>
+      <c r="F51" s="3" t="s">
+        <v>194</v>
+      </c>
+      <c r="G51" s="7">
+        <v>52.15</v>
       </c>
       <c r="H51" s="2">
-        <v>2</v>
-      </c>
-      <c r="I51" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="J51" s="1">
+        <v>3</v>
+      </c>
+      <c r="I51" s="6">
+        <v>651875</v>
+      </c>
+      <c r="J51" s="6">
+        <v>12500</v>
+      </c>
+      <c r="K51" s="1">
         <v>108</v>
       </c>
-      <c r="K51" s="2" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="52" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L51" s="2" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="52" spans="1:12" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A52" s="1" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B52" s="2" t="s">
-        <v>135</v>
+        <v>130</v>
       </c>
       <c r="C52" s="1">
         <v>111</v>
@@ -2919,31 +3130,34 @@
       <c r="E52" s="1">
         <v>160</v>
       </c>
-      <c r="F52" s="1" t="s">
-        <v>200</v>
-      </c>
-      <c r="G52" s="2">
-        <v>50</v>
+      <c r="F52" s="3" t="s">
+        <v>195</v>
+      </c>
+      <c r="G52" s="7">
+        <v>34.119999999999997</v>
       </c>
       <c r="H52" s="2">
         <v>2</v>
       </c>
-      <c r="I52" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="J52" s="1">
+      <c r="I52" s="6">
+        <v>446972</v>
+      </c>
+      <c r="J52" s="6">
+        <v>13100</v>
+      </c>
+      <c r="K52" s="1">
         <v>108</v>
       </c>
-      <c r="K52" s="2" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="53" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L52" s="2" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="53" spans="1:12" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A53" s="1" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B53" s="2" t="s">
-        <v>136</v>
+        <v>131</v>
       </c>
       <c r="C53" s="1">
         <v>112</v>
@@ -2954,31 +3168,34 @@
       <c r="E53" s="1">
         <v>111</v>
       </c>
-      <c r="F53" s="1" t="s">
-        <v>201</v>
-      </c>
-      <c r="G53" s="2">
-        <v>50</v>
+      <c r="F53" s="3" t="s">
+        <v>196</v>
+      </c>
+      <c r="G53" s="7">
+        <v>36.14</v>
       </c>
       <c r="H53" s="2">
         <v>2</v>
       </c>
-      <c r="I53" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="J53" s="1">
-        <v>111</v>
-      </c>
-      <c r="K53" s="2" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="54" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="I53" s="6">
+        <v>473434</v>
+      </c>
+      <c r="J53" s="6">
+        <v>13100</v>
+      </c>
+      <c r="K53" s="1">
+        <v>111</v>
+      </c>
+      <c r="L53" s="2" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="54" spans="1:12" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A54" s="1" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B54" s="2" t="s">
-        <v>137</v>
+        <v>132</v>
       </c>
       <c r="C54" s="1">
         <v>160</v>
@@ -2989,31 +3206,34 @@
       <c r="E54" s="1">
         <v>111</v>
       </c>
-      <c r="F54" s="1" t="s">
-        <v>202</v>
-      </c>
-      <c r="G54" s="2">
-        <v>50</v>
+      <c r="F54" s="3" t="s">
+        <v>197</v>
+      </c>
+      <c r="G54" s="7">
+        <v>79.78</v>
       </c>
       <c r="H54" s="2">
         <v>2</v>
       </c>
-      <c r="I54" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="J54" s="1">
+      <c r="I54" s="6">
+        <v>925448</v>
+      </c>
+      <c r="J54" s="6">
+        <v>11600</v>
+      </c>
+      <c r="K54" s="1">
         <v>5</v>
       </c>
-      <c r="K54" s="2" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="55" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L54" s="2" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="55" spans="1:12" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A55" s="1" t="s">
-        <v>152</v>
+        <v>147</v>
       </c>
       <c r="B55" s="2" t="s">
-        <v>156</v>
+        <v>151</v>
       </c>
       <c r="C55" s="1">
         <v>147</v>
@@ -3024,31 +3244,34 @@
       <c r="E55" s="1">
         <v>111</v>
       </c>
-      <c r="F55" s="1" t="s">
-        <v>203</v>
-      </c>
-      <c r="G55" s="2">
-        <v>50</v>
+      <c r="F55" s="3" t="s">
+        <v>198</v>
+      </c>
+      <c r="G55" s="7">
+        <v>82.71</v>
       </c>
       <c r="H55" s="2">
-        <v>2</v>
-      </c>
-      <c r="I55" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="J55" s="1">
+        <v>4</v>
+      </c>
+      <c r="I55" s="6">
+        <v>984249</v>
+      </c>
+      <c r="J55" s="6">
+        <v>11900</v>
+      </c>
+      <c r="K55" s="1">
         <v>107</v>
       </c>
-      <c r="K55" s="2" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="56" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L55" s="2" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="56" spans="1:12" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A56" s="1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B56" s="2" t="s">
-        <v>155</v>
+        <v>150</v>
       </c>
       <c r="C56" s="1">
         <v>181</v>
@@ -3059,31 +3282,34 @@
       <c r="E56" s="1">
         <v>111</v>
       </c>
-      <c r="F56" s="1" t="s">
-        <v>204</v>
-      </c>
-      <c r="G56" s="2">
-        <v>50</v>
+      <c r="F56" s="3" t="s">
+        <v>199</v>
+      </c>
+      <c r="G56" s="7">
+        <v>97.53</v>
       </c>
       <c r="H56" s="2">
-        <v>2</v>
-      </c>
-      <c r="I56" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="J56" s="1">
+        <v>3</v>
+      </c>
+      <c r="I56" s="6">
+        <v>1092336</v>
+      </c>
+      <c r="J56" s="6">
+        <v>11200</v>
+      </c>
+      <c r="K56" s="1">
         <v>78</v>
       </c>
-      <c r="K56" s="2" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="57" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L56" s="2" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="57" spans="1:12" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A57" s="1" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B57" s="2" t="s">
-        <v>138</v>
+        <v>133</v>
       </c>
       <c r="C57" s="1">
         <v>195</v>
@@ -3094,31 +3320,34 @@
       <c r="E57" s="1">
         <v>112</v>
       </c>
-      <c r="F57" s="1" t="s">
-        <v>205</v>
-      </c>
-      <c r="G57" s="2">
-        <v>50</v>
+      <c r="F57" s="3" t="s">
+        <v>200</v>
+      </c>
+      <c r="G57" s="7">
+        <v>88.21</v>
       </c>
       <c r="H57" s="2">
         <v>2</v>
       </c>
-      <c r="I57" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="J57" s="1">
+      <c r="I57" s="6">
+        <v>996773</v>
+      </c>
+      <c r="J57" s="6">
+        <v>11300</v>
+      </c>
+      <c r="K57" s="1">
         <v>79</v>
       </c>
-      <c r="K57" s="2" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="58" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L57" s="2" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="58" spans="1:12" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A58" s="1" t="s">
         <v>10</v>
       </c>
       <c r="B58" s="2" t="s">
-        <v>139</v>
+        <v>134</v>
       </c>
       <c r="C58" s="1">
         <v>195</v>
@@ -3129,31 +3358,34 @@
       <c r="E58" s="1">
         <v>223</v>
       </c>
-      <c r="F58" s="1" t="s">
-        <v>206</v>
-      </c>
-      <c r="G58" s="2">
-        <v>50</v>
+      <c r="F58" s="3" t="s">
+        <v>201</v>
+      </c>
+      <c r="G58" s="7">
+        <v>77.02</v>
       </c>
       <c r="H58" s="2">
         <v>2</v>
       </c>
-      <c r="I58" s="3">
-        <v>350000</v>
+      <c r="I58" s="6">
+        <v>901134</v>
       </c>
       <c r="J58" s="6">
+        <v>11700</v>
+      </c>
+      <c r="K58" s="4">
         <v>65</v>
       </c>
-      <c r="K58" s="2" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="59" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L58" s="2" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="59" spans="1:12" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A59" s="1" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B59" s="2" t="s">
-        <v>140</v>
+        <v>135</v>
       </c>
       <c r="C59" s="1">
         <v>181</v>
@@ -3164,31 +3396,34 @@
       <c r="E59" s="1">
         <v>223</v>
       </c>
-      <c r="F59" s="1" t="s">
-        <v>207</v>
-      </c>
-      <c r="G59" s="2">
+      <c r="F59" s="3" t="s">
+        <v>202</v>
+      </c>
+      <c r="G59" s="7">
+        <v>53.76</v>
+      </c>
+      <c r="H59" s="2">
+        <v>3</v>
+      </c>
+      <c r="I59" s="6">
+        <v>666624</v>
+      </c>
+      <c r="J59" s="6">
+        <v>12400</v>
+      </c>
+      <c r="K59" s="1">
         <v>50</v>
       </c>
-      <c r="H59" s="2">
-        <v>2</v>
-      </c>
-      <c r="I59" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="J59" s="1">
-        <v>50</v>
-      </c>
-      <c r="K59" s="2" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="60" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L59" s="2" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="60" spans="1:12" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A60" s="1" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B60" s="2" t="s">
-        <v>141</v>
+        <v>136</v>
       </c>
       <c r="C60" s="1">
         <v>160</v>
@@ -3199,31 +3434,34 @@
       <c r="E60" s="1">
         <v>224</v>
       </c>
-      <c r="F60" s="1" t="s">
-        <v>216</v>
-      </c>
-      <c r="G60" s="2">
-        <v>50</v>
+      <c r="F60" s="3" t="s">
+        <v>211</v>
+      </c>
+      <c r="G60" s="7">
+        <v>65.680000000000007</v>
       </c>
       <c r="H60" s="2">
-        <v>2</v>
-      </c>
-      <c r="I60" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="J60" s="1">
+        <v>1</v>
+      </c>
+      <c r="I60" s="6">
+        <v>794728</v>
+      </c>
+      <c r="J60" s="6">
+        <v>12100</v>
+      </c>
+      <c r="K60" s="1">
         <v>48</v>
       </c>
-      <c r="K60" s="2" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="61" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L60" s="2" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="61" spans="1:12" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A61" s="1" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B61" s="2" t="s">
-        <v>142</v>
+        <v>137</v>
       </c>
       <c r="C61" s="1">
         <v>112</v>
@@ -3234,31 +3472,34 @@
       <c r="E61" s="1">
         <v>223</v>
       </c>
-      <c r="F61" s="1" t="s">
-        <v>208</v>
-      </c>
-      <c r="G61" s="2">
-        <v>50</v>
+      <c r="F61" s="3" t="s">
+        <v>203</v>
+      </c>
+      <c r="G61" s="7">
+        <v>85.97</v>
       </c>
       <c r="H61" s="2">
         <v>2</v>
       </c>
-      <c r="I61" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="J61" s="1">
+      <c r="I61" s="6">
+        <v>971461</v>
+      </c>
+      <c r="J61" s="6">
+        <v>11300</v>
+      </c>
+      <c r="K61" s="1">
         <v>48</v>
       </c>
-      <c r="K61" s="2" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="62" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L61" s="2" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="62" spans="1:12" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A62" s="1" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B62" s="2" t="s">
-        <v>143</v>
+        <v>138</v>
       </c>
       <c r="C62" s="1">
         <v>111</v>
@@ -3269,31 +3510,34 @@
       <c r="E62" s="1">
         <v>224</v>
       </c>
-      <c r="F62" s="1" t="s">
-        <v>209</v>
-      </c>
-      <c r="G62" s="2">
-        <v>50</v>
+      <c r="F62" s="3" t="s">
+        <v>204</v>
+      </c>
+      <c r="G62" s="7">
+        <v>84.27</v>
       </c>
       <c r="H62" s="2">
         <v>2</v>
       </c>
-      <c r="I62" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="J62" s="1">
+      <c r="I62" s="6">
+        <v>952251</v>
+      </c>
+      <c r="J62" s="6">
+        <v>11300</v>
+      </c>
+      <c r="K62" s="1">
         <v>48</v>
       </c>
-      <c r="K62" s="2" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="63" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L62" s="2" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="63" spans="1:12" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A63" s="1" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B63" s="2" t="s">
-        <v>144</v>
+        <v>139</v>
       </c>
       <c r="C63" s="1">
         <v>111</v>
@@ -3304,31 +3548,34 @@
       <c r="E63" s="1">
         <v>223</v>
       </c>
-      <c r="F63" s="1" t="s">
-        <v>210</v>
-      </c>
-      <c r="G63" s="2">
-        <v>50</v>
+      <c r="F63" s="3" t="s">
+        <v>205</v>
+      </c>
+      <c r="G63" s="7">
+        <v>85.26</v>
       </c>
       <c r="H63" s="2">
         <v>2</v>
       </c>
-      <c r="I63" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="J63" s="1">
+      <c r="I63" s="6">
+        <v>963438</v>
+      </c>
+      <c r="J63" s="6">
+        <v>11300</v>
+      </c>
+      <c r="K63" s="1">
         <v>48</v>
       </c>
-      <c r="K63" s="2" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="64" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L63" s="2" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="64" spans="1:12" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A64" s="1" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B64" s="2" t="s">
-        <v>153</v>
+        <v>148</v>
       </c>
       <c r="C64" s="1">
         <v>181</v>
@@ -3339,31 +3586,34 @@
       <c r="E64" s="1">
         <v>255</v>
       </c>
-      <c r="F64" s="1" t="s">
-        <v>211</v>
-      </c>
-      <c r="G64" s="2">
-        <v>50</v>
+      <c r="F64" s="3" t="s">
+        <v>206</v>
+      </c>
+      <c r="G64" s="7">
+        <v>97.47</v>
       </c>
       <c r="H64" s="2">
         <v>2</v>
       </c>
-      <c r="I64" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="J64" s="1">
+      <c r="I64" s="6">
+        <v>1067296.5</v>
+      </c>
+      <c r="J64" s="6">
+        <v>10950</v>
+      </c>
+      <c r="K64" s="1">
         <v>25</v>
       </c>
-      <c r="K64" s="2" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="65" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L64" s="2" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="65" spans="1:12" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A65" s="1" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B65" s="2" t="s">
-        <v>154</v>
+        <v>149</v>
       </c>
       <c r="C65" s="1">
         <v>111</v>
@@ -3374,31 +3624,34 @@
       <c r="E65" s="1">
         <v>223</v>
       </c>
-      <c r="F65" s="1" t="s">
-        <v>212</v>
-      </c>
-      <c r="G65" s="2">
-        <v>50</v>
+      <c r="F65" s="3" t="s">
+        <v>207</v>
+      </c>
+      <c r="G65" s="7">
+        <v>89.19</v>
       </c>
       <c r="H65" s="2">
         <v>2</v>
       </c>
-      <c r="I65" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="J65" s="1">
+      <c r="I65" s="6">
+        <v>1061361</v>
+      </c>
+      <c r="J65" s="6">
+        <v>11900</v>
+      </c>
+      <c r="K65" s="1">
         <v>15</v>
       </c>
-      <c r="K65" s="2" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="66" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L65" s="2" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="66" spans="1:12" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A66" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B66" s="2" t="s">
-        <v>146</v>
+        <v>141</v>
       </c>
       <c r="C66" s="1">
         <v>223</v>
@@ -3409,31 +3662,34 @@
       <c r="E66" s="1">
         <v>206</v>
       </c>
-      <c r="F66" s="1" t="s">
-        <v>213</v>
-      </c>
-      <c r="G66" s="2">
-        <v>50</v>
+      <c r="F66" s="3" t="s">
+        <v>208</v>
+      </c>
+      <c r="G66" s="7">
+        <v>79.599999999999994</v>
       </c>
       <c r="H66" s="2">
         <v>2</v>
       </c>
-      <c r="I66" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="J66" s="1">
+      <c r="I66" s="6">
+        <v>923360</v>
+      </c>
+      <c r="J66" s="6">
+        <v>11600</v>
+      </c>
+      <c r="K66" s="1">
         <v>105</v>
       </c>
-      <c r="K66" s="2" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="67" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L66" s="2" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="67" spans="1:12" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A67" s="1" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B67" s="2" t="s">
-        <v>147</v>
+        <v>142</v>
       </c>
       <c r="C67" s="1">
         <v>223</v>
@@ -3444,31 +3700,34 @@
       <c r="E67" s="1">
         <v>215</v>
       </c>
-      <c r="F67" s="1" t="s">
-        <v>214</v>
-      </c>
-      <c r="G67" s="2">
-        <v>50</v>
+      <c r="F67" s="3" t="s">
+        <v>209</v>
+      </c>
+      <c r="G67" s="7">
+        <v>76.459999999999994</v>
       </c>
       <c r="H67" s="2">
         <v>2</v>
       </c>
-      <c r="I67" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="J67" s="1">
+      <c r="I67" s="6">
+        <v>894582</v>
+      </c>
+      <c r="J67" s="6">
+        <v>11700</v>
+      </c>
+      <c r="K67" s="1">
         <v>108</v>
       </c>
-      <c r="K67" s="2" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="68" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L67" s="2" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="68" spans="1:12" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A68" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B68" s="2" t="s">
-        <v>148</v>
+        <v>143</v>
       </c>
       <c r="C68" s="1">
         <v>223</v>
@@ -3479,31 +3738,34 @@
       <c r="E68" s="1">
         <v>224</v>
       </c>
-      <c r="F68" s="1" t="s">
-        <v>215</v>
-      </c>
-      <c r="G68" s="2">
-        <v>50</v>
+      <c r="F68" s="3" t="s">
+        <v>210</v>
+      </c>
+      <c r="G68" s="7">
+        <v>34.11</v>
       </c>
       <c r="H68" s="2">
-        <v>2</v>
-      </c>
-      <c r="I68" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="J68" s="1">
+        <v>1</v>
+      </c>
+      <c r="I68" s="6">
+        <v>450252</v>
+      </c>
+      <c r="J68" s="6">
+        <v>13200</v>
+      </c>
+      <c r="K68" s="1">
         <v>109</v>
       </c>
-      <c r="K68" s="2" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="69" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L68" s="2" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="69" spans="1:12" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A69" s="1" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B69" s="2" t="s">
-        <v>145</v>
+        <v>140</v>
       </c>
       <c r="C69" s="1">
         <v>216</v>
@@ -3514,31 +3776,34 @@
       <c r="E69" s="1">
         <v>223</v>
       </c>
-      <c r="F69" s="1" t="s">
-        <v>217</v>
-      </c>
-      <c r="G69" s="2">
-        <v>50</v>
+      <c r="F69" s="3" t="s">
+        <v>212</v>
+      </c>
+      <c r="G69" s="7">
+        <v>62.51</v>
       </c>
       <c r="H69" s="2">
-        <v>2</v>
-      </c>
-      <c r="I69" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="I69" s="6">
+        <v>756371</v>
+      </c>
+      <c r="J69" s="6">
+        <v>12100</v>
+      </c>
+      <c r="K69" s="1">
+        <v>113</v>
+      </c>
+      <c r="L69" s="2" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="70" spans="1:12" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A70" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="J69" s="1">
-        <v>113</v>
-      </c>
-      <c r="K69" s="2" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="70" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A70" s="1" t="s">
-        <v>12</v>
-      </c>
       <c r="B70" s="2" t="s">
-        <v>149</v>
+        <v>144</v>
       </c>
       <c r="C70" s="1">
         <v>206</v>
@@ -3549,37 +3814,51 @@
       <c r="E70" s="1">
         <v>224</v>
       </c>
-      <c r="F70" s="1" t="s">
-        <v>218</v>
-      </c>
-      <c r="G70" s="2">
-        <v>50</v>
+      <c r="F70" s="3" t="s">
+        <v>213</v>
+      </c>
+      <c r="G70" s="7">
+        <v>82.62</v>
       </c>
       <c r="H70" s="2">
         <v>2</v>
       </c>
-      <c r="I70" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="J70" s="1">
+      <c r="I70" s="6">
+        <v>950130</v>
+      </c>
+      <c r="J70" s="6">
+        <v>11500</v>
+      </c>
+      <c r="K70" s="1">
         <v>79</v>
       </c>
-      <c r="K70" s="2" t="s">
-        <v>80</v>
+      <c r="L70" s="2" t="s">
+        <v>145</v>
       </c>
     </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:K70">
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:L70">
     <sortCondition ref="B2:B70"/>
   </sortState>
+  <conditionalFormatting sqref="L2:L70">
+    <cfRule type="cellIs" dxfId="2" priority="1" operator="equal">
+      <formula>"Rezerwacja"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="1" priority="2" operator="equal">
+      <formula>"Sprzedane"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="0" priority="3" operator="equal">
+      <formula>"Dostępne"</formula>
+    </cfRule>
+  </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="K2:K70" xr:uid="{63A27076-74EE-4804-9509-D0975931E98A}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="L2:L70" xr:uid="{63A27076-74EE-4804-9509-D0975931E98A}">
       <formula1>"Dostępne,Rezerwacja,Sprzedane"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError sqref="K1 A1:I1" numberStoredAsText="1"/>
+    <ignoredError sqref="L1 A1:H1" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Nowy styl dla aplikacji
</commit_message>
<xml_diff>
--- a/mieszkania.xlsx
+++ b/mieszkania.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mateu\Desktop\BlockViewDesktop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9D090802-9B8D-47C2-8043-BEE33BE5C256}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{37936523-B618-4082-90A2-1078B1B47C4D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-90" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Mieszkania" sheetId="1" r:id="rId1"/>
@@ -685,7 +685,7 @@
     <t>static\karty-lokali\R101\R101_16_L.pdf</t>
   </si>
   <si>
-    <t>price/meter</t>
+    <t>price_meter</t>
   </si>
 </sst>
 </file>
@@ -758,29 +758,25 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="3" fontId="2" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="3" fontId="2" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="2" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="164" fontId="2" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left"/>
       <protection locked="0"/>
     </xf>
@@ -788,7 +784,7 @@
   <cellStyles count="1">
     <cellStyle name="Normalny" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="6">
+  <dxfs count="3">
     <dxf>
       <font>
         <color rgb="FF00B050"/>
@@ -802,21 +798,6 @@
     <dxf>
       <font>
         <color rgb="FFFFC000"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FFFF0000"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF00B050"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF00B050"/>
       </font>
     </dxf>
   </dxfs>
@@ -1233,7 +1214,7 @@
       <c r="F2" s="3" t="s">
         <v>152</v>
       </c>
-      <c r="G2" s="7">
+      <c r="G2" s="2">
         <v>75.13</v>
       </c>
       <c r="H2" s="2">
@@ -1271,7 +1252,7 @@
       <c r="F3" s="3" t="s">
         <v>153</v>
       </c>
-      <c r="G3" s="7">
+      <c r="G3" s="2">
         <v>53.66</v>
       </c>
       <c r="H3" s="2">
@@ -1309,7 +1290,7 @@
       <c r="F4" s="3" t="s">
         <v>154</v>
       </c>
-      <c r="G4" s="7">
+      <c r="G4" s="2">
         <v>40.520000000000003</v>
       </c>
       <c r="H4" s="2">
@@ -1347,7 +1328,7 @@
       <c r="F5" s="3" t="s">
         <v>155</v>
       </c>
-      <c r="G5" s="7">
+      <c r="G5" s="2">
         <v>56.4</v>
       </c>
       <c r="H5" s="2">
@@ -1385,7 +1366,7 @@
       <c r="F6" s="3" t="s">
         <v>156</v>
       </c>
-      <c r="G6" s="7">
+      <c r="G6" s="2">
         <v>56.4</v>
       </c>
       <c r="H6" s="2">
@@ -1423,7 +1404,7 @@
       <c r="F7" s="3" t="s">
         <v>157</v>
       </c>
-      <c r="G7" s="7">
+      <c r="G7" s="2">
         <v>37.409999999999997</v>
       </c>
       <c r="H7" s="2">
@@ -1461,7 +1442,7 @@
       <c r="F8" s="3" t="s">
         <v>158</v>
       </c>
-      <c r="G8" s="7">
+      <c r="G8" s="2">
         <v>64.209999999999994</v>
       </c>
       <c r="H8" s="2">
@@ -1499,7 +1480,7 @@
       <c r="F9" s="3" t="s">
         <v>159</v>
       </c>
-      <c r="G9" s="7">
+      <c r="G9" s="2">
         <v>53.48</v>
       </c>
       <c r="H9" s="2">
@@ -1537,7 +1518,7 @@
       <c r="F10" s="3" t="s">
         <v>160</v>
       </c>
-      <c r="G10" s="7">
+      <c r="G10" s="2">
         <v>55.63</v>
       </c>
       <c r="H10" s="2">
@@ -1575,7 +1556,7 @@
       <c r="F11" s="3" t="s">
         <v>161</v>
       </c>
-      <c r="G11" s="7">
+      <c r="G11" s="2">
         <v>66.87</v>
       </c>
       <c r="H11" s="2">
@@ -1613,7 +1594,7 @@
       <c r="F12" s="3" t="s">
         <v>162</v>
       </c>
-      <c r="G12" s="7">
+      <c r="G12" s="2">
         <v>74.23</v>
       </c>
       <c r="H12" s="2">
@@ -1651,7 +1632,7 @@
       <c r="F13" s="3" t="s">
         <v>163</v>
       </c>
-      <c r="G13" s="7">
+      <c r="G13" s="2">
         <v>56.42</v>
       </c>
       <c r="H13" s="2">
@@ -1689,7 +1670,7 @@
       <c r="F14" s="3" t="s">
         <v>164</v>
       </c>
-      <c r="G14" s="7">
+      <c r="G14" s="2">
         <v>54.93</v>
       </c>
       <c r="H14" s="2">
@@ -1727,7 +1708,7 @@
       <c r="F15" s="3" t="s">
         <v>165</v>
       </c>
-      <c r="G15" s="7">
+      <c r="G15" s="2">
         <v>37.4</v>
       </c>
       <c r="H15" s="2">
@@ -1765,7 +1746,7 @@
       <c r="F16" s="3" t="s">
         <v>166</v>
       </c>
-      <c r="G16" s="7">
+      <c r="G16" s="2">
         <v>35.950000000000003</v>
       </c>
       <c r="H16" s="2">
@@ -1803,7 +1784,7 @@
       <c r="F17" s="3" t="s">
         <v>167</v>
       </c>
-      <c r="G17" s="7">
+      <c r="G17" s="2">
         <v>54.47</v>
       </c>
       <c r="H17" s="2">
@@ -1841,7 +1822,7 @@
       <c r="F18" s="3" t="s">
         <v>168</v>
       </c>
-      <c r="G18" s="7">
+      <c r="G18" s="2">
         <v>66.45</v>
       </c>
       <c r="H18" s="2">
@@ -1879,7 +1860,7 @@
       <c r="F19" s="3" t="s">
         <v>169</v>
       </c>
-      <c r="G19" s="7">
+      <c r="G19" s="2">
         <v>74.39</v>
       </c>
       <c r="H19" s="2">
@@ -1917,7 +1898,7 @@
       <c r="F20" s="3" t="s">
         <v>170</v>
       </c>
-      <c r="G20" s="7">
+      <c r="G20" s="2">
         <v>75.319999999999993</v>
       </c>
       <c r="H20" s="2">
@@ -1955,7 +1936,7 @@
       <c r="F21" s="3" t="s">
         <v>171</v>
       </c>
-      <c r="G21" s="7">
+      <c r="G21" s="2">
         <v>53.66</v>
       </c>
       <c r="H21" s="2">
@@ -1993,7 +1974,7 @@
       <c r="F22" s="3" t="s">
         <v>172</v>
       </c>
-      <c r="G22" s="7">
+      <c r="G22" s="2">
         <v>40.520000000000003</v>
       </c>
       <c r="H22" s="2">
@@ -2031,7 +2012,7 @@
       <c r="F23" s="3" t="s">
         <v>173</v>
       </c>
-      <c r="G23" s="7">
+      <c r="G23" s="2">
         <v>56.4</v>
       </c>
       <c r="H23" s="2">
@@ -2069,7 +2050,7 @@
       <c r="F24" s="3" t="s">
         <v>174</v>
       </c>
-      <c r="G24" s="7">
+      <c r="G24" s="2">
         <v>56.4</v>
       </c>
       <c r="H24" s="2">
@@ -2107,7 +2088,7 @@
       <c r="F25" s="3" t="s">
         <v>175</v>
       </c>
-      <c r="G25" s="7">
+      <c r="G25" s="2">
         <v>58.86</v>
       </c>
       <c r="H25" s="2">
@@ -2145,7 +2126,7 @@
       <c r="F26" s="3" t="s">
         <v>176</v>
       </c>
-      <c r="G26" s="7">
+      <c r="G26" s="2">
         <v>60.69</v>
       </c>
       <c r="H26" s="2">
@@ -2183,7 +2164,7 @@
       <c r="F27" s="3" t="s">
         <v>214</v>
       </c>
-      <c r="G27" s="7">
+      <c r="G27" s="2">
         <v>50.49</v>
       </c>
       <c r="H27" s="2">
@@ -2221,7 +2202,7 @@
       <c r="F28" s="3" t="s">
         <v>215</v>
       </c>
-      <c r="G28" s="7">
+      <c r="G28" s="2">
         <v>52.48</v>
       </c>
       <c r="H28" s="2">
@@ -2259,7 +2240,7 @@
       <c r="F29" s="3" t="s">
         <v>177</v>
       </c>
-      <c r="G29" s="7">
+      <c r="G29" s="2">
         <v>67.05</v>
       </c>
       <c r="H29" s="2">
@@ -2297,7 +2278,7 @@
       <c r="F30" s="3" t="s">
         <v>178</v>
       </c>
-      <c r="G30" s="7">
+      <c r="G30" s="2">
         <v>74.23</v>
       </c>
       <c r="H30" s="2">
@@ -2335,7 +2316,7 @@
       <c r="F31" s="3" t="s">
         <v>216</v>
       </c>
-      <c r="G31" s="7">
+      <c r="G31" s="2">
         <v>52.61</v>
       </c>
       <c r="H31" s="2">
@@ -2373,7 +2354,7 @@
       <c r="F32" s="3" t="s">
         <v>217</v>
       </c>
-      <c r="G32" s="7">
+      <c r="G32" s="2">
         <v>52.15</v>
       </c>
       <c r="H32" s="2">
@@ -2411,7 +2392,7 @@
       <c r="F33" s="3" t="s">
         <v>218</v>
       </c>
-      <c r="G33" s="7">
+      <c r="G33" s="2">
         <v>33.83</v>
       </c>
       <c r="H33" s="2">
@@ -2449,7 +2430,7 @@
       <c r="F34" s="3" t="s">
         <v>219</v>
       </c>
-      <c r="G34" s="7">
+      <c r="G34" s="2">
         <v>35.950000000000003</v>
       </c>
       <c r="H34" s="2">
@@ -2487,7 +2468,7 @@
       <c r="F35" s="3" t="s">
         <v>220</v>
       </c>
-      <c r="G35" s="7">
+      <c r="G35" s="2">
         <v>51.58</v>
       </c>
       <c r="H35" s="2">
@@ -2525,7 +2506,7 @@
       <c r="F36" s="3" t="s">
         <v>179</v>
       </c>
-      <c r="G36" s="7">
+      <c r="G36" s="2">
         <v>66.66</v>
       </c>
       <c r="H36" s="2">
@@ -2563,7 +2544,7 @@
       <c r="F37" s="3" t="s">
         <v>180</v>
       </c>
-      <c r="G37" s="7">
+      <c r="G37" s="2">
         <v>93.93</v>
       </c>
       <c r="H37" s="2">
@@ -2601,7 +2582,7 @@
       <c r="F38" s="3" t="s">
         <v>181</v>
       </c>
-      <c r="G38" s="7">
+      <c r="G38" s="2">
         <v>75.19</v>
       </c>
       <c r="H38" s="2">
@@ -2639,7 +2620,7 @@
       <c r="F39" s="3" t="s">
         <v>182</v>
       </c>
-      <c r="G39" s="7">
+      <c r="G39" s="2">
         <v>53.66</v>
       </c>
       <c r="H39" s="2">
@@ -2677,7 +2658,7 @@
       <c r="F40" s="3" t="s">
         <v>183</v>
       </c>
-      <c r="G40" s="7">
+      <c r="G40" s="2">
         <v>40.57</v>
       </c>
       <c r="H40" s="2">
@@ -2715,7 +2696,7 @@
       <c r="F41" s="3" t="s">
         <v>184</v>
       </c>
-      <c r="G41" s="7">
+      <c r="G41" s="2">
         <v>56.43</v>
       </c>
       <c r="H41" s="2">
@@ -2753,7 +2734,7 @@
       <c r="F42" s="3" t="s">
         <v>185</v>
       </c>
-      <c r="G42" s="7">
+      <c r="G42" s="2">
         <v>56.43</v>
       </c>
       <c r="H42" s="2">
@@ -2791,7 +2772,7 @@
       <c r="F43" s="3" t="s">
         <v>186</v>
       </c>
-      <c r="G43" s="7">
+      <c r="G43" s="2">
         <v>58.87</v>
       </c>
       <c r="H43" s="2">
@@ -2829,7 +2810,7 @@
       <c r="F44" s="3" t="s">
         <v>187</v>
       </c>
-      <c r="G44" s="7">
+      <c r="G44" s="2">
         <v>60.77</v>
       </c>
       <c r="H44" s="2">
@@ -2867,7 +2848,7 @@
       <c r="F45" s="3" t="s">
         <v>188</v>
       </c>
-      <c r="G45" s="7">
+      <c r="G45" s="2">
         <v>50.49</v>
       </c>
       <c r="H45" s="2">
@@ -2905,7 +2886,7 @@
       <c r="F46" s="3" t="s">
         <v>189</v>
       </c>
-      <c r="G46" s="7">
+      <c r="G46" s="2">
         <v>80.790000000000006</v>
       </c>
       <c r="H46" s="2">
@@ -2943,7 +2924,7 @@
       <c r="F47" s="3" t="s">
         <v>190</v>
       </c>
-      <c r="G47" s="7">
+      <c r="G47" s="2">
         <v>81.7</v>
       </c>
       <c r="H47" s="2">
@@ -2981,7 +2962,7 @@
       <c r="F48" s="3" t="s">
         <v>191</v>
       </c>
-      <c r="G48" s="7">
+      <c r="G48" s="2">
         <v>99.02</v>
       </c>
       <c r="H48" s="2">
@@ -3019,7 +3000,7 @@
       <c r="F49" s="3" t="s">
         <v>192</v>
       </c>
-      <c r="G49" s="7">
+      <c r="G49" s="2">
         <v>57.32</v>
       </c>
       <c r="H49" s="2">
@@ -3057,7 +3038,7 @@
       <c r="F50" s="3" t="s">
         <v>193</v>
       </c>
-      <c r="G50" s="7">
+      <c r="G50" s="2">
         <v>52.54</v>
       </c>
       <c r="H50" s="2">
@@ -3095,7 +3076,7 @@
       <c r="F51" s="3" t="s">
         <v>194</v>
       </c>
-      <c r="G51" s="7">
+      <c r="G51" s="2">
         <v>52.15</v>
       </c>
       <c r="H51" s="2">
@@ -3133,7 +3114,7 @@
       <c r="F52" s="3" t="s">
         <v>195</v>
       </c>
-      <c r="G52" s="7">
+      <c r="G52" s="2">
         <v>34.119999999999997</v>
       </c>
       <c r="H52" s="2">
@@ -3171,7 +3152,7 @@
       <c r="F53" s="3" t="s">
         <v>196</v>
       </c>
-      <c r="G53" s="7">
+      <c r="G53" s="2">
         <v>36.14</v>
       </c>
       <c r="H53" s="2">
@@ -3209,7 +3190,7 @@
       <c r="F54" s="3" t="s">
         <v>197</v>
       </c>
-      <c r="G54" s="7">
+      <c r="G54" s="2">
         <v>79.78</v>
       </c>
       <c r="H54" s="2">
@@ -3247,7 +3228,7 @@
       <c r="F55" s="3" t="s">
         <v>198</v>
       </c>
-      <c r="G55" s="7">
+      <c r="G55" s="2">
         <v>82.71</v>
       </c>
       <c r="H55" s="2">
@@ -3285,7 +3266,7 @@
       <c r="F56" s="3" t="s">
         <v>199</v>
       </c>
-      <c r="G56" s="7">
+      <c r="G56" s="2">
         <v>97.53</v>
       </c>
       <c r="H56" s="2">
@@ -3323,7 +3304,7 @@
       <c r="F57" s="3" t="s">
         <v>200</v>
       </c>
-      <c r="G57" s="7">
+      <c r="G57" s="2">
         <v>88.21</v>
       </c>
       <c r="H57" s="2">
@@ -3361,7 +3342,7 @@
       <c r="F58" s="3" t="s">
         <v>201</v>
       </c>
-      <c r="G58" s="7">
+      <c r="G58" s="2">
         <v>77.02</v>
       </c>
       <c r="H58" s="2">
@@ -3399,7 +3380,7 @@
       <c r="F59" s="3" t="s">
         <v>202</v>
       </c>
-      <c r="G59" s="7">
+      <c r="G59" s="2">
         <v>53.76</v>
       </c>
       <c r="H59" s="2">
@@ -3437,7 +3418,7 @@
       <c r="F60" s="3" t="s">
         <v>211</v>
       </c>
-      <c r="G60" s="7">
+      <c r="G60" s="2">
         <v>65.680000000000007</v>
       </c>
       <c r="H60" s="2">
@@ -3475,7 +3456,7 @@
       <c r="F61" s="3" t="s">
         <v>203</v>
       </c>
-      <c r="G61" s="7">
+      <c r="G61" s="2">
         <v>85.97</v>
       </c>
       <c r="H61" s="2">
@@ -3513,7 +3494,7 @@
       <c r="F62" s="3" t="s">
         <v>204</v>
       </c>
-      <c r="G62" s="7">
+      <c r="G62" s="2">
         <v>84.27</v>
       </c>
       <c r="H62" s="2">
@@ -3551,7 +3532,7 @@
       <c r="F63" s="3" t="s">
         <v>205</v>
       </c>
-      <c r="G63" s="7">
+      <c r="G63" s="2">
         <v>85.26</v>
       </c>
       <c r="H63" s="2">
@@ -3589,7 +3570,7 @@
       <c r="F64" s="3" t="s">
         <v>206</v>
       </c>
-      <c r="G64" s="7">
+      <c r="G64" s="2">
         <v>97.47</v>
       </c>
       <c r="H64" s="2">
@@ -3627,7 +3608,7 @@
       <c r="F65" s="3" t="s">
         <v>207</v>
       </c>
-      <c r="G65" s="7">
+      <c r="G65" s="2">
         <v>89.19</v>
       </c>
       <c r="H65" s="2">
@@ -3665,7 +3646,7 @@
       <c r="F66" s="3" t="s">
         <v>208</v>
       </c>
-      <c r="G66" s="7">
+      <c r="G66" s="2">
         <v>79.599999999999994</v>
       </c>
       <c r="H66" s="2">
@@ -3703,7 +3684,7 @@
       <c r="F67" s="3" t="s">
         <v>209</v>
       </c>
-      <c r="G67" s="7">
+      <c r="G67" s="2">
         <v>76.459999999999994</v>
       </c>
       <c r="H67" s="2">
@@ -3741,7 +3722,7 @@
       <c r="F68" s="3" t="s">
         <v>210</v>
       </c>
-      <c r="G68" s="7">
+      <c r="G68" s="2">
         <v>34.11</v>
       </c>
       <c r="H68" s="2">
@@ -3779,7 +3760,7 @@
       <c r="F69" s="3" t="s">
         <v>212</v>
       </c>
-      <c r="G69" s="7">
+      <c r="G69" s="2">
         <v>62.51</v>
       </c>
       <c r="H69" s="2">
@@ -3817,7 +3798,7 @@
       <c r="F70" s="3" t="s">
         <v>213</v>
       </c>
-      <c r="G70" s="7">
+      <c r="G70" s="2">
         <v>82.62</v>
       </c>
       <c r="H70" s="2">

</xml_diff>